<commit_message>
Prepare release 1.0.0 (#171)
* prepare release 1.0.0

* change sequence 3ba6b25cc3a4df5009773e0ba27a967730070432
</commit_message>
<xml_diff>
--- a/main/ig/CodeSystem-as-cs-intern-id-systems.xlsx
+++ b/main/ig/CodeSystem-as-cs-intern-id-systems.xlsx
@@ -30,7 +30,7 @@
     <t>Version</t>
   </si>
   <si>
-    <t>1.0.0-ballot-4</t>
+    <t>1.0.0</t>
   </si>
   <si>
     <t>Name</t>
@@ -57,7 +57,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2024-04-02T14:01:28+00:00</t>
+    <t>2024-04-03T13:55:00+00:00</t>
   </si>
   <si>
     <t>Publisher</t>

</xml_diff>

<commit_message>
Add release notes and publication request for first snapshot (#217)
* add release notes and publication request for first snapshot

* Update release-notes.md edfd65ca744e0bf7d687f7f0ae33173612afab48
</commit_message>
<xml_diff>
--- a/main/ig/CodeSystem-as-cs-intern-id-systems.xlsx
+++ b/main/ig/CodeSystem-as-cs-intern-id-systems.xlsx
@@ -30,7 +30,7 @@
     <t>Version</t>
   </si>
   <si>
-    <t>1.0.1</t>
+    <t>1.1.0-snapshot</t>
   </si>
   <si>
     <t>Name</t>
@@ -57,7 +57,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2024-07-10T09:54:14+00:00</t>
+    <t>2024-07-10T10:00:25+00:00</t>
   </si>
   <si>
     <t>Publisher</t>

</xml_diff>

<commit_message>
Mise à jour de FrCore dans sushi-config (#219)
* update sushi-config

* update mapping & release note b2ec087a7a9bb68b47430578da77b2b522b6b7ef
</commit_message>
<xml_diff>
--- a/main/ig/CodeSystem-as-cs-intern-id-systems.xlsx
+++ b/main/ig/CodeSystem-as-cs-intern-id-systems.xlsx
@@ -30,7 +30,7 @@
     <t>Version</t>
   </si>
   <si>
-    <t>1.1.0-snapshot</t>
+    <t>1.1.0-snapshot-2</t>
   </si>
   <si>
     <t>Name</t>
@@ -57,7 +57,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2024-07-11T14:20:03+00:00</t>
+    <t>2024-07-11T15:32:47+00:00</t>
   </si>
   <si>
     <t>Publisher</t>

</xml_diff>